<commit_message>
Add $11,600 Alexis contractor payment to buildout total
Treats Cesar's confirmed cash/transfer to Alexis for the contractor as
buildout, assumed additive to Amex FNR charges pending overlap confirm.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/amex-buildout-classified.xlsx
+++ b/finance/amex-buildout-classified.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="BuildoutSummary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AllLines" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="BuildoutOnly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ManualAdjustments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="AllLines" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BuildoutOnly" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AllLines'!$A$1:$K$127</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BuildoutOnly'!$A$1:$K$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllLines'!$A$1:$K$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'BuildoutOnly'!$A$1:$K$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -118,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -140,6 +141,8 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -505,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -560,11 +563,11 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>33578.03</v>
+        <v>45178.03</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Merchant clearly shop build/setup</t>
+          <t>Amex Yes + manual contractor $11,600 (assumed additive to Amex FNR)</t>
         </is>
       </c>
     </row>
@@ -575,7 +578,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>33705.39</v>
+        <v>45305.39</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -631,7 +634,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BUILDOUT BY CATEGORY (Yes only)</t>
+          <t>BUILDOUT BY CATEGORY (Yes + manual)</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -665,11 +668,11 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Flooring / paint / finishes</t>
+          <t>Construction / contractor / permits</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>11845.69</v>
+        <v>15950</v>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
@@ -683,11 +686,11 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Waiting area / furniture</t>
+          <t>Flooring / paint / finishes</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>6299.73</v>
+        <v>11845.69</v>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
@@ -701,11 +704,11 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Construction / contractor / permits</t>
+          <t>Waiting area / furniture</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>4350</v>
+        <v>6299.73</v>
       </c>
     </row>
     <row r="17">
@@ -758,6 +761,10 @@
         <v>1035.33</v>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -772,9 +779,24 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Manual add</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>$11,600 to Alexis for contractor. Amex already shows FNR $4,350 ($2,000 Cesar + $2,350 Alexis). Current model treats $11,600 as EXTRA. If the $11,600 was the total contractor budget and already covers those Amex charges, true added cash is $11,600 − $4,350 = $7,250 — tell me and I'll switch.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A29:E29"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
@@ -788,7 +810,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K127"/>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+      <c r="D1" s="17" t="inlineStr">
+        <is>
+          <t>Buildout?</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>Who / how paid</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="H1" s="17" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I1" s="17" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>2026-02/03 (approx)</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>11600</v>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Buildout</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Construction / contractor / permits</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>Alexis (cash/transfer to pay contractor)</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>Cash/transfer so Alexis can pay contractor</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>Cesar confirmed $11,600 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $11,600 already includes those Amex hits.</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>manual-cesar</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>MANUAL-ALEXIS-CONTRACTOR-11600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7775,19 +7913,70 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="18" t="inlineStr">
+        <is>
+          <t>2026-02/03 (approx)</t>
+        </is>
+      </c>
+      <c r="B128" s="6" t="n">
+        <v>11600</v>
+      </c>
+      <c r="C128" s="18" t="inlineStr">
+        <is>
+          <t>Buildout</t>
+        </is>
+      </c>
+      <c r="D128" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E128" s="18" t="inlineStr">
+        <is>
+          <t>Construction / contractor / permits</t>
+        </is>
+      </c>
+      <c r="F128" s="18" t="inlineStr">
+        <is>
+          <t>Alexis (cash/transfer to pay contractor)</t>
+        </is>
+      </c>
+      <c r="G128" s="18" t="inlineStr">
+        <is>
+          <t>Cash/transfer so Alexis can pay contractor</t>
+        </is>
+      </c>
+      <c r="H128" s="18" t="inlineStr">
+        <is>
+          <t>Cesar confirmed $11,600 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $11,600 already includes those Amex hits.</t>
+        </is>
+      </c>
+      <c r="I128" s="18" t="inlineStr"/>
+      <c r="J128" s="18" t="inlineStr">
+        <is>
+          <t>manual-cesar</t>
+        </is>
+      </c>
+      <c r="K128" s="18" t="inlineStr">
+        <is>
+          <t>MANUAL-ALEXIS-CONTRACTOR-11600</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12480,6 +12669,57 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="18" t="inlineStr">
+        <is>
+          <t>2026-02/03 (approx)</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="n">
+        <v>11600</v>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>Buildout</t>
+        </is>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Construction / contractor / permits</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="inlineStr">
+        <is>
+          <t>Alexis (cash/transfer to pay contractor)</t>
+        </is>
+      </c>
+      <c r="G86" s="18" t="inlineStr">
+        <is>
+          <t>Cash/transfer so Alexis can pay contractor</t>
+        </is>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>Cesar confirmed $11,600 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $11,600 already includes those Amex hits.</t>
+        </is>
+      </c>
+      <c r="I86" s="18" t="inlineStr"/>
+      <c r="J86" s="18" t="inlineStr">
+        <is>
+          <t>manual-cesar</t>
+        </is>
+      </c>
+      <c r="K86" s="18" t="inlineStr">
+        <is>
+          <t>MANUAL-ALEXIS-CONTRACTOR-11600</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Model $11,600 Alexis contractor cost as 50/50 partner split
Keeps full amount in buildout totals; adds ContractorSplit sheet showing
each partner owes $5,800 economically and the true-up if Cesar fronted it.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/amex-buildout-classified.xlsx
+++ b/finance/amex-buildout-classified.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="BuildoutSummary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ManualAdjustments" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AllLines" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="BuildoutOnly" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ContractorSplit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ManualAdjustments" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AllLines" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BuildoutOnly" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllLines'!$A$1:$K$127</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'BuildoutOnly'!$A$1:$K$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllLines'!$A$1:$K$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BuildoutOnly'!$A$1:$K$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +49,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="9">
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,6 +149,7 @@
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -761,10 +768,6 @@
         <v>1035.33</v>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -782,14 +785,14 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Manual add</t>
+          <t>Manual add — $11,600 contractor SPLIT 50/50</t>
         </is>
       </c>
     </row>
     <row r="29" ht="70" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>$11,600 to Alexis for contractor. Amex already shows FNR $4,350 ($2,000 Cesar + $2,350 Alexis). Current model treats $11,600 as EXTRA. If the $11,600 was the total contractor budget and already covers those Amex charges, true added cash is $11,600 − $4,350 = $7,250 — tell me and I'll switch.</t>
+          <t>Total buildout still includes full $45,178.03. The $11,600 Alexis contractor payment is split 50/50 → Cesar $5,800 / Partner $5,800. See ContractorSplit sheet. If Cesar fronted all $11,600, Partner owes Cesar $5,800.</t>
         </is>
       </c>
     </row>
@@ -810,6 +813,296 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Alexis contractor $11,600 — 50/50 split</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cesar: "half of it… we splitting that." Shop still recognizes full $11,600 as buildout cost; economically each partner owns half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Total to Alexis for contractor</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>11600</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Full buildout cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Cesar share (50%)</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>His half of that bill</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Partner share (50%)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Their half of that bill</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>If Cesar fronted the full $11,600 → Partner owes Cesar</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>True-up check</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>If they each already put in $5,800 → true-up</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Even — no cash owed on this line</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Related Amex FNR charges (already in Amex buildout)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>FNR on Amex — Cesar card</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>02/12 AplPay FNR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>FNR on Amex — Alexis card</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>2350</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>03/05 FNR Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Amex FNR subtotal</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>4350</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Still counted in Amex buildout Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Buildout picture with this rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Total shop buildout (Amex Yes + $11,600)</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>45178.03</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Cost of building the shop</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Of the $11,600 — Cesar economic share</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Of the $11,600 — Partner economic share</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Likely Partner → Cesar true-up on this line</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>5800</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Only if Cesar fronted all $11,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Still need: who actually sent Alexis the $11,600 (Cesar alone, both, or shop account)? That decides whether Partner owes Cesar $5,800 on this line.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -891,7 +1184,7 @@
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>Alexis (cash/transfer to pay contractor)</t>
+          <t>Split 50/50 (Cesar $5,800 / Partner $5,800)</t>
         </is>
       </c>
       <c r="G2" s="12" t="inlineStr">
@@ -901,7 +1194,7 @@
       </c>
       <c r="H2" s="12" t="inlineStr">
         <is>
-          <t>Cesar confirmed $11,600 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $11,600 already includes those Amex hits.</t>
+          <t>TOTAL contractor cash/transfer via Alexis = $11,600. SPLIT 50/50: Cesar $5,800 / Partner $5,800. Who fronted the $11,600 still matters for true-up (if Cesar fronted all, Partner owes Cesar $5,800).</t>
         </is>
       </c>
       <c r="I2" s="12" t="inlineStr">
@@ -920,7 +1213,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7970,7 +8263,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Reconcile Cesar buildout list to paper $29,835 and $13.8k contractor
Adds a reconciliation workbook from Cesar's Amex/Chase/cash/deposit/t-shirt
and contractor figures, and updates contractor total to $13,800 split 50/50.

Co-authored-by: cesarblendss-ai <cesarblendss-ai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/finance/amex-buildout-classified.xlsx
+++ b/finance/amex-buildout-classified.xlsx
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>45178.03</v>
+        <v>47378.03</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>45305.39</v>
+        <v>47505.39</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>15950</v>
+        <v>18150</v>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
@@ -768,6 +768,10 @@
         <v>1035.33</v>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -813,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -824,17 +828,18 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Alexis contractor $11,600 — 50/50 split</t>
+          <t>Alexis contractor $13,800 — 50/50 split</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cesar: "half of it… we splitting that." Shop still recognizes full $11,600 as buildout cost; economically each partner owns half.</t>
-        </is>
-      </c>
-    </row>
+          <t>Cesar: "half of it… we splitting that." Shop still recognizes full $13,800 as buildout cost; economically each partner owns half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -859,7 +864,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>11600</v>
+        <v>13800</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -874,7 +879,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>5800</v>
+        <v>6900</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -889,7 +894,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>5800</v>
+        <v>6900</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -900,11 +905,11 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>If Cesar fronted the full $11,600 → Partner owes Cesar</t>
+          <t>If Cesar fronted the full $13,800 → Partner owes Cesar</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>5800</v>
+        <v>6900</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -915,7 +920,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>If they each already put in $5,800 → true-up</t>
+          <t>If they each already put in $6,900 → true-up</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
@@ -927,6 +932,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -996,6 +1002,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -1023,7 +1030,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Total shop buildout (Amex Yes + $11,600)</t>
+          <t>Total shop buildout (Amex Yes + $13,800)</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
@@ -1038,11 +1045,11 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Of the $11,600 — Cesar economic share</t>
+          <t>Of the $13,800 — Cesar economic share</t>
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>5800</v>
+        <v>6900</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
@@ -1053,11 +1060,11 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Of the $11,600 — Partner economic share</t>
+          <t>Of the $13,800 — Partner economic share</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>5800</v>
+        <v>6900</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -1072,21 +1079,28 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>5800</v>
+        <v>6900</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Only if Cesar fronted all $11,600</t>
-        </is>
-      </c>
-    </row>
+          <t>Only if Cesar fronted all $13,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Still need: who actually sent Alexis the $11,600 (Cesar alone, both, or shop account)? That decides whether Partner owes Cesar $5,800 on this line.</t>
-        </is>
-      </c>
-    </row>
+          <t>Still need: who actually sent Alexis the $13,800 (Cesar alone, both, or shop account)? That decides whether Partner owes Cesar $6,900 on this line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
@@ -1103,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1165,7 +1179,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>11600</v>
+        <v>13800</v>
       </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
@@ -1184,7 +1198,7 @@
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>Split 50/50 (Cesar $5,800 / Partner $5,800)</t>
+          <t>Split 50/50 (Cesar $6,900 / Partner $6,900)</t>
         </is>
       </c>
       <c r="G2" s="12" t="inlineStr">
@@ -1194,7 +1208,7 @@
       </c>
       <c r="H2" s="12" t="inlineStr">
         <is>
-          <t>TOTAL contractor cash/transfer via Alexis = $11,600. SPLIT 50/50: Cesar $5,800 / Partner $5,800. Who fronted the $11,600 still matters for true-up (if Cesar fronted all, Partner owes Cesar $5,800).</t>
+          <t>TOTAL contractor cash/transfer via Alexis = $11,600. SPLIT 50/50: Cesar $6,900 / Partner $6,900. Who fronted the $11,600 still matters for true-up (if Cesar fronted all, Partner owes Cesar $6,900).</t>
         </is>
       </c>
       <c r="I2" s="12" t="inlineStr">
@@ -1204,7 +1218,7 @@
       </c>
       <c r="J2" s="12" t="inlineStr">
         <is>
-          <t>MANUAL-ALEXIS-CONTRACTOR-11600</t>
+          <t>MANUAL-ALEXIS-CONTRACTOR-13800</t>
         </is>
       </c>
     </row>
@@ -8213,7 +8227,7 @@
         </is>
       </c>
       <c r="B128" s="6" t="n">
-        <v>11600</v>
+        <v>13800</v>
       </c>
       <c r="C128" s="18" t="inlineStr">
         <is>
@@ -8242,7 +8256,7 @@
       </c>
       <c r="H128" s="18" t="inlineStr">
         <is>
-          <t>Cesar confirmed $11,600 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $11,600 already includes those Amex hits.</t>
+          <t>Cesar confirmed $13,800 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $13,800 already includes those Amex hits.</t>
         </is>
       </c>
       <c r="I128" s="18" t="inlineStr"/>
@@ -8253,7 +8267,7 @@
       </c>
       <c r="K128" s="18" t="inlineStr">
         <is>
-          <t>MANUAL-ALEXIS-CONTRACTOR-11600</t>
+          <t>MANUAL-ALEXIS-CONTRACTOR-13800</t>
         </is>
       </c>
     </row>
@@ -12969,7 +12983,7 @@
         </is>
       </c>
       <c r="B86" s="6" t="n">
-        <v>11600</v>
+        <v>13800</v>
       </c>
       <c r="C86" s="18" t="inlineStr">
         <is>
@@ -12998,7 +13012,7 @@
       </c>
       <c r="H86" s="18" t="inlineStr">
         <is>
-          <t>Cesar confirmed $11,600 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $11,600 already includes those Amex hits.</t>
+          <t>Cesar confirmed $13,800 for Alexis → contractor. Assumed IN ADDITION to Amex FNR charges ($2,000 Cesar + $2,350 Alexis = $4,350). Change if $13,800 already includes those Amex hits.</t>
         </is>
       </c>
       <c r="I86" s="18" t="inlineStr"/>
@@ -13009,7 +13023,7 @@
       </c>
       <c r="K86" s="18" t="inlineStr">
         <is>
-          <t>MANUAL-ALEXIS-CONTRACTOR-11600</t>
+          <t>MANUAL-ALEXIS-CONTRACTOR-13800</t>
         </is>
       </c>
     </row>

</xml_diff>